<commit_message>
Updated Books Management page
</commit_message>
<xml_diff>
--- a/transactions.xlsx
+++ b/transactions.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,28 +484,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>546b2d8</t>
+          <t>546B2D6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>22ir200</t>
+          <t>23uree044</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46196.95561342593</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>46197.64907407408</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>46197.64916666667</v>
+      </c>
       <c r="F2" s="3" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Issued</t>
+          <t>Returned</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -515,28 +517,30 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4v6b7n</t>
+          <t>546B2D6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22ECE002</t>
+          <t>23uree14</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>46196.95494212963</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>46197.63337962963</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>46197.63347222222</v>
+      </c>
       <c r="F3" s="3" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Issued</t>
+          <t>Returned</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -546,20 +550,20 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A4V6N7</t>
+          <t>546b2d8</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>22ECE001</t>
+          <t>22ir200</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>46196.9116087963</v>
+        <v>46196.95561342593</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="3" t="n">
@@ -577,30 +581,28 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>546B2D6</t>
+          <t>4v6b7n</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23uree44</t>
+          <t>22ECE002</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>46196.90346064815</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>46196.90355324074</v>
-      </c>
+        <v>46196.95494212963</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Returned</t>
+          <t>Issued</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -610,30 +612,28 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>8ED85A6</t>
+          <t>A4V6N7</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23uree44</t>
+          <t>22ECE001</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46196.6021875</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>46196.68454861111</v>
-      </c>
+        <v>46196.9116087963</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Returned</t>
+          <t>Issued</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -643,28 +643,30 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">8ed85a6	</t>
+          <t>546B2D6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>98657</t>
+          <t>23uree44</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>46191.47747685185</v>
-      </c>
-      <c r="E7" t="inlineStr"/>
+        <v>46196.90346064815</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46196.90355324074</v>
+      </c>
       <c r="F7" s="3" t="n">
-        <v>46206</v>
+        <v>46211</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Issued</t>
+          <t>Returned</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -674,26 +676,26 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>546b2d6</t>
+          <t>8ED85A6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>980858</t>
+          <t>23uree44</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46191.47686342592</v>
+        <v>46196.6021875</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46196.68800925926</v>
+        <v>46196.68454861111</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>46206</v>
+        <v>46211</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -707,30 +709,28 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>546b2d6</t>
+          <t xml:space="preserve">8ed85a6	</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>980858</t>
+          <t>98657</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46188.67393518519</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>46196.68818287037</v>
-      </c>
+        <v>46191.47747685185</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Returned</t>
+          <t>Issued</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -740,7 +740,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -749,17 +749,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>95667789</t>
+          <t>980858</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46185.70017361111</v>
+        <v>46191.47686342592</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>46185.7003125</v>
+        <v>46196.68800925926</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>46200</v>
+        <v>46206</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -773,28 +773,30 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4v6b7n</t>
+          <t>546b2d6</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23uree044</t>
+          <t>980858</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46185.56961805555</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
+        <v>46188.67393518519</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>46196.68818287037</v>
+      </c>
       <c r="F11" s="3" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Issued</t>
+          <t>Returned</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -804,7 +806,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -813,14 +815,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23uree14</t>
+          <t>95667789</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>46185.50045138889</v>
+        <v>46185.70017361111</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>46185.50056712963</v>
+        <v>46185.7003125</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>46200</v>
@@ -837,30 +839,28 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>aa11</t>
+          <t>4v6b7n</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>bb22</t>
+          <t>23uree044</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>46182.86261574074</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>46185.53834490741</v>
-      </c>
+        <v>46185.56961805555</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>46197</v>
+        <v>46200</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Returned</t>
+          <t>Issued</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -870,11 +870,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2346780</t>
+          <t>546b2d6</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -883,15 +883,17 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>46182.62140046297</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
+        <v>46185.50045138889</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>46185.50056712963</v>
+      </c>
       <c r="F14" s="3" t="n">
-        <v>46197</v>
+        <v>46200</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Issued</t>
+          <t>Returned</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -901,23 +903,23 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>546b2d6</t>
+          <t>aa11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23uree044</t>
+          <t>bb22</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>46182.61601851852</v>
+        <v>46182.86261574074</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>46182.62153935185</v>
+        <v>46185.53834490741</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>46197</v>
@@ -934,20 +936,20 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3457ui</t>
+          <t>2346780</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>56789</t>
+          <t>23uree14</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>46182.61335648148</v>
+        <v>46182.62140046297</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" s="3" t="n">
@@ -965,11 +967,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>8ed85a6</t>
+          <t>546b2d6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -978,10 +980,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>46182.61320601852</v>
+        <v>46182.61601851852</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>46196.68547453704</v>
+        <v>46182.62153935185</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>46197</v>
@@ -995,6 +997,70 @@
         <v>0</v>
       </c>
       <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>3457ui</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>56789</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>46182.61335648148</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" s="3" t="n">
+        <v>46197</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Issued</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>8ed85a6</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23uree044</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>46182.61320601852</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>46196.68547453704</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>46197</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Returned</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>